<commit_message>
feat: add V3P post-plateau probes and reporting updates
</commit_message>
<xml_diff>
--- a/docs/00-规范与记录/实验记录表.xlsx
+++ b/docs/00-规范与记录/实验记录表.xlsx
@@ -73,6 +73,7 @@
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -93,74 +94,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
 </styleSheet>
 </file>
 
@@ -563,7 +496,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T152"/>
+  <dimension ref="A1:T171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -14322,6 +14255,1602 @@
         </is>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>V3P-G-57-PGradKernelAttn_seed1</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>V3P-G-57-PGradKernelAttn</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_path_g</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>V3P 路径 G：G2-b 壁面 ∇p kernel attention head</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="J153" t="n">
+        <v>1</v>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N153" t="n">
+        <v>0.4204</v>
+      </c>
+      <c r="O153" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P153" t="n">
+        <v>0.928</v>
+      </c>
+      <c r="Q153" t="n">
+        <v>103</v>
+      </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_g2b_pgrad_kernel_attn_wall13000_near2000_split_AG_v1_seed1_20260606_142906</t>
+        </is>
+      </c>
+      <c r="T153" t="inlineStr">
+        <is>
+          <t>No-Go jobs 5410/5437/5438；三 seed 0.392–0.420；未超 AsymW-a 4957</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>V3P-G-57-PGradKernelAttn_seed3</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>V3P-G-57-PGradKernelAttn</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_path_g</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>V3P 路径 G：G2-b 壁面 ∇p kernel attention head</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="J154" t="n">
+        <v>3</v>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N154" t="n">
+        <v>0.3986</v>
+      </c>
+      <c r="O154" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P154" t="n">
+        <v>0.9514</v>
+      </c>
+      <c r="Q154" t="n">
+        <v>130</v>
+      </c>
+      <c r="R154" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_g2b_pgrad_kernel_attn_wall13000_near2000_split_AG_v1_seed3_20260607_115628</t>
+        </is>
+      </c>
+      <c r="T154" t="inlineStr">
+        <is>
+          <t>No-Go jobs 5410/5437/5438；三 seed 0.392–0.420；未超 AsymW-a 4957</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>V3P-G-Baseline-AsymW-a_seed1</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>V3P-G-Baseline-AsymW-a</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_path_g</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>V3P 路径 G：post-denylist AsymW-a 同 split 基线</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="J155" t="n">
+        <v>1</v>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N155" t="n">
+        <v>0.4341</v>
+      </c>
+      <c r="O155" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P155" t="n">
+        <v>0.9238</v>
+      </c>
+      <c r="Q155" t="n">
+        <v>165</v>
+      </c>
+      <c r="R155" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260607_115628</t>
+        </is>
+      </c>
+      <c r="T155" t="inlineStr">
+        <is>
+          <t>基线 job 5439；best_wss wss=0.434（post-denylist 对照）</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>V3P-G-57-PGradKernelAttn_seed2</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>V3P-G-57-PGradKernelAttn</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_path_g</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>V3P 路径 G：G2-b 壁面 ∇p kernel attention head</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="J156" t="n">
+        <v>2</v>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N156" t="n">
+        <v>0.3923</v>
+      </c>
+      <c r="O156" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P156" t="n">
+        <v>0.9379</v>
+      </c>
+      <c r="Q156" t="n">
+        <v>136</v>
+      </c>
+      <c r="R156" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_g2b_pgrad_kernel_attn_wall13000_near2000_split_AG_v1_seed2_20260607_115628</t>
+        </is>
+      </c>
+      <c r="T156" t="inlineStr">
+        <is>
+          <t>No-Go jobs 5410/5437/5438；三 seed 0.392–0.420；未超 AsymW-a 4957</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>V3P-G-54a-VNHeadPlain_seed1</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>V3P-G-54a-VNHeadPlain</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_path_g</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>V3P 路径 G：G1 向量归一化 head 纯结构 Probe</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="J157" t="n">
+        <v>1</v>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N157" t="n">
+        <v>0.427</v>
+      </c>
+      <c r="O157" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P157" t="n">
+        <v>0.9433</v>
+      </c>
+      <c r="Q157" t="n">
+        <v>141</v>
+      </c>
+      <c r="R157" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_g1a_vnhead_plain_wall13000_near2000_split_AG_v1_seed1_20260607_123105</t>
+        </is>
+      </c>
+      <c r="T157" t="inlineStr">
+        <is>
+          <t>No-Go job 5425；best_wss wss=0.427≈基线 band</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>V3P-G-Baseline-AsymW-a-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>V3P-G-Baseline-AsymW-a-post5463</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_path_g</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>V3P 路径 G/I：post5463 graphs 无 SSL 基线 band</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="J158" t="n">
+        <v>1</v>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N158" t="n">
+        <v>0.4278</v>
+      </c>
+      <c r="O158" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P158" t="n">
+        <v>0.9256</v>
+      </c>
+      <c r="Q158" t="n">
+        <v>185</v>
+      </c>
+      <c r="R158" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260608_154606</t>
+        </is>
+      </c>
+      <c r="T158" t="inlineStr">
+        <is>
+          <t>三 seed 5466/5468/5478；band 0.409–0.437（均值 ~0.425）</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>V3P-G-Baseline-AsymW-a-post5463_seed2</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>V3P-G-Baseline-AsymW-a-post5463</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_path_g</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>V3P 路径 G/I：post5463 graphs 无 SSL 基线 band</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="J159" t="n">
+        <v>2</v>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N159" t="n">
+        <v>0.4374</v>
+      </c>
+      <c r="O159" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P159" t="n">
+        <v>0.9143</v>
+      </c>
+      <c r="Q159" t="n">
+        <v>86</v>
+      </c>
+      <c r="R159" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed2_20260608_154606</t>
+        </is>
+      </c>
+      <c r="T159" t="inlineStr">
+        <is>
+          <t>三 seed 5466/5468/5478；band 0.409–0.437（均值 ~0.425）</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>V3P-G-58-SSL-Finetune_seed1</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>V3P-G-58-SSL-Finetune</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_path_g</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>V3P 路径 G：G3 SSL 预训练 encoder 微调</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="J160" t="n">
+        <v>1</v>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N160" t="n">
+        <v>0.4401</v>
+      </c>
+      <c r="O160" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P160" t="n">
+        <v>0.9243</v>
+      </c>
+      <c r="Q160" t="n">
+        <v>98</v>
+      </c>
+      <c r="R160" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260609_124213</t>
+        </is>
+      </c>
+      <c r="T160" t="inlineStr">
+        <is>
+          <t>No-Go jobs 5474/5475；wss 0.435–0.440；未达 Go +0.03 vs post5463 band</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>V3P-G-58-SSL-Finetune_seed2</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>V3P-G-58-SSL-Finetune</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_path_g</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>V3P 路径 G：G3 SSL 预训练 encoder 微调</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="J161" t="n">
+        <v>2</v>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N161" t="n">
+        <v>0.4354</v>
+      </c>
+      <c r="O161" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P161" t="n">
+        <v>0.927</v>
+      </c>
+      <c r="Q161" t="n">
+        <v>164</v>
+      </c>
+      <c r="R161" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed2_20260609_124213</t>
+        </is>
+      </c>
+      <c r="T161" t="inlineStr">
+        <is>
+          <t>No-Go jobs 5474/5475；wss 0.435–0.440；未达 Go +0.03 vs post5463 band</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>V3P-G-Baseline-AsymW-a-post5463_seed3</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>V3P-G-Baseline-AsymW-a-post5463</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_path_g</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>V3P 路径 G/I：post5463 graphs 无 SSL 基线 band</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="J162" t="n">
+        <v>3</v>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N162" t="n">
+        <v>0.4087</v>
+      </c>
+      <c r="O162" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P162" t="n">
+        <v>0.9423</v>
+      </c>
+      <c r="Q162" t="n">
+        <v>131</v>
+      </c>
+      <c r="R162" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed3_20260610_003850</t>
+        </is>
+      </c>
+      <c r="T162" t="inlineStr">
+        <is>
+          <t>三 seed 5466/5468/5478；band 0.409–0.437（均值 ~0.425）</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>V3P-I2-PC-Intrinsic_seed1</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>V3P-I2-PC-Intrinsic</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_path_i</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>V3P 路径 I：I2-PC 本征坐标 WSS 4 维 local frame</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="J163" t="n">
+        <v>1</v>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N163" t="n">
+        <v>0.4175</v>
+      </c>
+      <c r="O163" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P163" t="n">
+        <v>0.9319</v>
+      </c>
+      <c r="Q163" t="n">
+        <v>109</v>
+      </c>
+      <c r="R163" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_i2pc_intrinsic_geom_pw_asymw_wall13000_near2000_split_AG_v1_seed1_20260618_143615</t>
+        </is>
+      </c>
+      <c r="T163" t="inlineStr">
+        <is>
+          <t>No-Go job 5741；best_wss wss=0.417；local frame 4D 未破 band</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>V3P-I6-diag-AsymW-a-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>V3P-I6-diag-AsymW-a-post5463</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_path_i</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>V3P 路径 I：I6 梯度/训练动力学诊断（200ep）</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="J164" t="n">
+        <v>1</v>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N164" t="n">
+        <v>0.4286</v>
+      </c>
+      <c r="O164" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P164" t="n">
+        <v>0.9298</v>
+      </c>
+      <c r="Q164" t="n">
+        <v>163</v>
+      </c>
+      <c r="R164" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_i6diag_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260619_174001</t>
+        </is>
+      </c>
+      <c r="T164" t="inlineStr">
+        <is>
+          <t>平台期带宽参考 job 5463/I6-diag；best_wss wss=0.429 · r2_p=0.930</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>V3P-I6-a-AsymW-a-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>V3P-I6-a-AsymW-a-post5463</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_path_i</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>V3P 路径 I/M-E：I6-a 两阶段冻结 best_wss 探针</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="J165" t="n">
+        <v>1</v>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N165" t="n">
+        <v>0.4457</v>
+      </c>
+      <c r="O165" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P165" t="n">
+        <v>0.9407</v>
+      </c>
+      <c r="Q165" t="n">
+        <v>33</v>
+      </c>
+      <c r="R165" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_i6a_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260625_154438</t>
+        </is>
+      </c>
+      <c r="T165" t="inlineStr">
+        <is>
+          <t>Go job 5810；best_wss wss=0.446（+0.017 vs I6-diag）；未扩 seed</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>V3P-M-E-WSSOnly-AsymW-a-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>V3P-M-E-WSSOnly-AsymW-a-post5463</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_m_e</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>V3P M-E：WSS-only（λ_p=0）上限探针</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="J166" t="n">
+        <v>1</v>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N166" t="n">
+        <v>0.4105</v>
+      </c>
+      <c r="O166" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P166" t="n">
+        <v>-0.4092</v>
+      </c>
+      <c r="Q166" t="n">
+        <v>13</v>
+      </c>
+      <c r="R166" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_mewssonly_localpool_main01_geom_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260625_155102</t>
+        </is>
+      </c>
+      <c r="T166" t="inlineStr">
+        <is>
+          <t>No-Go job 5811；WSS-only；wss=0.411 但 r2_p≈−0.41</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>V3P-M-E-PWeak-AsymW-a-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>V3P-M-E-PWeak-AsymW-a-post5463</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_m_e</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>V3P M-E：压力 λ 降 5× 弱压力探针</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="J167" t="n">
+        <v>1</v>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N167" t="n">
+        <v>0.4112</v>
+      </c>
+      <c r="O167" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P167" t="n">
+        <v>0.9463</v>
+      </c>
+      <c r="Q167" t="n">
+        <v>151</v>
+      </c>
+      <c r="R167" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_mepweak_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260625_155102</t>
+        </is>
+      </c>
+      <c r="T167" t="inlineStr">
+        <is>
+          <t>No-Go job 5812；弱压力 λ；best_wss wss=0.411</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>V3P-M-E-EJ-PGradBridge-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>V3P-M-E-EJ-PGradBridge-post5463</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_me_ej</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>V3P M-E：E-J 压力梯度桥接 rich pgrad GPU probe</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="J168" t="n">
+        <v>1</v>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N168" t="n">
+        <v>0.4009</v>
+      </c>
+      <c r="O168" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P168" t="n">
+        <v>0.9355</v>
+      </c>
+      <c r="Q168" t="n">
+        <v>77</v>
+      </c>
+      <c r="R168" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_me_ej_pgradbridge_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260629_154517</t>
+        </is>
+      </c>
+      <c r="T168" t="inlineStr">
+        <is>
+          <t>No-Go job 5854；rich pgrad context；best_wss wss=0.401</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>V3P-J4-V3Dlite-MixedProbe-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>V3P-J4-V3Dlite-MixedProbe-post5463</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_platform_j</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>V3P 平台期：V3D-lite +1 病例 MixedProbe</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>split_AG_v3lite_v1</t>
+        </is>
+      </c>
+      <c r="J169" t="n">
+        <v>1</v>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N169" t="n">
+        <v>0.4231</v>
+      </c>
+      <c r="O169" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P169" t="n">
+        <v>0.9347</v>
+      </c>
+      <c r="Q169" t="n">
+        <v>39</v>
+      </c>
+      <c r="R169" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_j4v3dlite_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v3lite_v1_seed1_20260630_131820</t>
+        </is>
+      </c>
+      <c r="T169" t="inlineStr">
+        <is>
+          <t>No-Go job 5872；+1 ZHAO；best_wss wss=0.423（Δi6 −0.006）</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>V3P-J5-ActiveData-MixedProbe-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>V3P-J5-ActiveData-MixedProbe-post5463</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_platform_j</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>V3P 平台期：主动选数 +6 AAA MixedProbe</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>split_AG_active_v2_j5</t>
+        </is>
+      </c>
+      <c r="J170" t="n">
+        <v>1</v>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N170" t="n">
+        <v>0.433</v>
+      </c>
+      <c r="O170" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P170" t="n">
+        <v>0.9509</v>
+      </c>
+      <c r="Q170" t="n">
+        <v>37</v>
+      </c>
+      <c r="R170" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_j5activedata_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_active_v2_j5_seed1_20260701_002549</t>
+        </is>
+      </c>
+      <c r="T170" t="inlineStr">
+        <is>
+          <t>弱 No-Go jobs 5881–5883；+6 AAA；wss=0.433（Δi6 +0.004）；Go 0.459 未过</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>V3P-K1-BranchFeat-MixedProbe-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>V3P-K1-BranchFeat-MixedProbe-post5463</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>field</t>
+        </is>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>v3_pointcloud_path_k1</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>V3P 后平台期：K1 branch 拓扑特征 GPU 短训</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>AG_v1</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="J171" t="n">
+        <v>1</v>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_g01_wall</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>wss_r2_wss</t>
+        </is>
+      </c>
+      <c r="N171" t="n">
+        <v>0.3998</v>
+      </c>
+      <c r="O171" t="inlineStr">
+        <is>
+          <t>R2_p</t>
+        </is>
+      </c>
+      <c r="P171" t="n">
+        <v>0.9247</v>
+      </c>
+      <c r="Q171" t="n">
+        <v>29</v>
+      </c>
+      <c r="R171" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_k1branchfeat_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260701_150937</t>
+        </is>
+      </c>
+      <c r="T171" t="inlineStr">
+        <is>
+          <t>No-Go job 5886；branch 特征短训；best_wss wss=0.400（低于 I6-diag）</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14408,7 +15937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BF152"/>
+  <dimension ref="A1:BF171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -39315,6 +40844,2505 @@
         </is>
       </c>
     </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>V3P-G-57-PGradKernelAttn_seed1</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>V3P-G-57-PGradKernelAttn</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>1</v>
+      </c>
+      <c r="D153" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K153" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="N153" t="n">
+        <v>103</v>
+      </c>
+      <c r="O153" t="n">
+        <v>1.178787085002863</v>
+      </c>
+      <c r="P153" t="n">
+        <v>1.321895384441374</v>
+      </c>
+      <c r="Q153" t="n">
+        <v>1.3722824998007</v>
+      </c>
+      <c r="R153" t="n">
+        <v>2.240559345945638</v>
+      </c>
+      <c r="S153" t="n">
+        <v>0.05486642540481998</v>
+      </c>
+      <c r="T153" t="n">
+        <v>0.02871376028806584</v>
+      </c>
+      <c r="U153" t="n">
+        <v>-3.4332275390625e-05</v>
+      </c>
+      <c r="V153" t="n">
+        <v>-0.0002698898315429688</v>
+      </c>
+      <c r="W153" t="n">
+        <v>-2.348423004150391e-05</v>
+      </c>
+      <c r="X153" t="n">
+        <v>-0.06322883513760225</v>
+      </c>
+      <c r="Y153" t="n">
+        <v>0.9423441290855408</v>
+      </c>
+      <c r="Z153" t="n">
+        <v>0.4203905463218689</v>
+      </c>
+      <c r="AA153" t="n">
+        <v>0.6950980373573861</v>
+      </c>
+      <c r="AB153" t="n">
+        <v>0.03637051582336426</v>
+      </c>
+      <c r="AC153" t="n">
+        <v>0.01146304607391357</v>
+      </c>
+      <c r="AD153" t="n">
+        <v>0.3891435861587524</v>
+      </c>
+      <c r="AG153" t="n">
+        <v>36</v>
+      </c>
+      <c r="AH153" t="n">
+        <v>0.4684716463088989</v>
+      </c>
+      <c r="BE153" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_g2b_pgrad_kernel_attn_wall13000_near2000_split_AG_v1_seed1_20260606_142906</t>
+        </is>
+      </c>
+      <c r="BF153" t="inlineStr">
+        <is>
+          <t>No-Go jobs 5410/5437/5438；三 seed 0.392–0.420；未超 AsymW-a 4957</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>V3P-G-57-PGradKernelAttn_seed3</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>V3P-G-57-PGradKernelAttn</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>3</v>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K154" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="N154" t="n">
+        <v>130</v>
+      </c>
+      <c r="O154" t="n">
+        <v>1.178787085002863</v>
+      </c>
+      <c r="P154" t="n">
+        <v>1.321895384441374</v>
+      </c>
+      <c r="Q154" t="n">
+        <v>1.3722824998007</v>
+      </c>
+      <c r="R154" t="n">
+        <v>2.240559345945638</v>
+      </c>
+      <c r="S154" t="n">
+        <v>0.04939155661487634</v>
+      </c>
+      <c r="T154" t="n">
+        <v>0.02711568930041152</v>
+      </c>
+      <c r="U154" t="n">
+        <v>-3.4332275390625e-05</v>
+      </c>
+      <c r="V154" t="n">
+        <v>-0.0002698898315429688</v>
+      </c>
+      <c r="W154" t="n">
+        <v>-2.348423004150391e-05</v>
+      </c>
+      <c r="X154" t="n">
+        <v>-0.06322883513760225</v>
+      </c>
+      <c r="Y154" t="n">
+        <v>0.9532764554023743</v>
+      </c>
+      <c r="Z154" t="n">
+        <v>0.3985642194747925</v>
+      </c>
+      <c r="AA154" t="n">
+        <v>0.7080647440074185</v>
+      </c>
+      <c r="AB154" t="n">
+        <v>0.02422982454299927</v>
+      </c>
+      <c r="AC154" t="n">
+        <v>-0.005811691284179688</v>
+      </c>
+      <c r="AD154" t="n">
+        <v>0.3658928275108337</v>
+      </c>
+      <c r="AG154" t="n">
+        <v>114</v>
+      </c>
+      <c r="AH154" t="n">
+        <v>0.5041960477828979</v>
+      </c>
+      <c r="BE154" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_g2b_pgrad_kernel_attn_wall13000_near2000_split_AG_v1_seed3_20260607_115628</t>
+        </is>
+      </c>
+      <c r="BF154" t="inlineStr">
+        <is>
+          <t>No-Go jobs 5410/5437/5438；三 seed 0.392–0.420；未超 AsymW-a 4957</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>V3P-G-Baseline-AsymW-a_seed1</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>V3P-G-Baseline-AsymW-a</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>1</v>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K155" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="N155" t="n">
+        <v>165</v>
+      </c>
+      <c r="O155" t="n">
+        <v>1.178787085002863</v>
+      </c>
+      <c r="P155" t="n">
+        <v>1.321895384441374</v>
+      </c>
+      <c r="Q155" t="n">
+        <v>1.3722824998007</v>
+      </c>
+      <c r="R155" t="n">
+        <v>2.240559345945638</v>
+      </c>
+      <c r="S155" t="n">
+        <v>0.05256981712219286</v>
+      </c>
+      <c r="T155" t="n">
+        <v>0.02747472672325103</v>
+      </c>
+      <c r="U155" t="n">
+        <v>-3.4332275390625e-05</v>
+      </c>
+      <c r="V155" t="n">
+        <v>-0.0002698898315429688</v>
+      </c>
+      <c r="W155" t="n">
+        <v>-2.348423004150391e-05</v>
+      </c>
+      <c r="X155" t="n">
+        <v>-0.06322883513760225</v>
+      </c>
+      <c r="Y155" t="n">
+        <v>0.9470698833465576</v>
+      </c>
+      <c r="Z155" t="n">
+        <v>0.4341221451759338</v>
+      </c>
+      <c r="AA155" t="n">
+        <v>0.6868148792525859</v>
+      </c>
+      <c r="AB155" t="n">
+        <v>0.0003687739372253418</v>
+      </c>
+      <c r="AC155" t="n">
+        <v>0.004342436790466309</v>
+      </c>
+      <c r="AD155" t="n">
+        <v>0.400339663028717</v>
+      </c>
+      <c r="AG155" t="n">
+        <v>13</v>
+      </c>
+      <c r="AH155" t="n">
+        <v>0.4741111397743225</v>
+      </c>
+      <c r="BE155" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260607_115628</t>
+        </is>
+      </c>
+      <c r="BF155" t="inlineStr">
+        <is>
+          <t>基线 job 5439；best_wss wss=0.434（post-denylist 对照）</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>V3P-G-57-PGradKernelAttn_seed2</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>V3P-G-57-PGradKernelAttn</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>2</v>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K156" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="N156" t="n">
+        <v>136</v>
+      </c>
+      <c r="O156" t="n">
+        <v>1.178787085002863</v>
+      </c>
+      <c r="P156" t="n">
+        <v>1.321895384441374</v>
+      </c>
+      <c r="Q156" t="n">
+        <v>1.3722824998007</v>
+      </c>
+      <c r="R156" t="n">
+        <v>2.240559345945638</v>
+      </c>
+      <c r="S156" t="n">
+        <v>0.04745240442552821</v>
+      </c>
+      <c r="T156" t="n">
+        <v>0.02559356835133745</v>
+      </c>
+      <c r="U156" t="n">
+        <v>-3.4332275390625e-05</v>
+      </c>
+      <c r="V156" t="n">
+        <v>-0.0002698898315429688</v>
+      </c>
+      <c r="W156" t="n">
+        <v>-2.348423004150391e-05</v>
+      </c>
+      <c r="X156" t="n">
+        <v>-0.06322883513760225</v>
+      </c>
+      <c r="Y156" t="n">
+        <v>0.9568732380867004</v>
+      </c>
+      <c r="Z156" t="n">
+        <v>0.3923023343086243</v>
+      </c>
+      <c r="AA156" t="n">
+        <v>0.7117412215600707</v>
+      </c>
+      <c r="AB156" t="n">
+        <v>0.00373154878616333</v>
+      </c>
+      <c r="AC156" t="n">
+        <v>0.01475375890731812</v>
+      </c>
+      <c r="AD156" t="n">
+        <v>0.3847154378890991</v>
+      </c>
+      <c r="AG156" t="n">
+        <v>50</v>
+      </c>
+      <c r="AH156" t="n">
+        <v>0.501511812210083</v>
+      </c>
+      <c r="BE156" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_g2b_pgrad_kernel_attn_wall13000_near2000_split_AG_v1_seed2_20260607_115628</t>
+        </is>
+      </c>
+      <c r="BF156" t="inlineStr">
+        <is>
+          <t>No-Go jobs 5410/5437/5438；三 seed 0.392–0.420；未超 AsymW-a 4957</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>V3P-G-54a-VNHeadPlain_seed1</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>V3P-G-54a-VNHeadPlain</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>1</v>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K157" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="N157" t="n">
+        <v>141</v>
+      </c>
+      <c r="O157" t="n">
+        <v>1.178787085002863</v>
+      </c>
+      <c r="P157" t="n">
+        <v>1.321895384441374</v>
+      </c>
+      <c r="Q157" t="n">
+        <v>1.3722824998007</v>
+      </c>
+      <c r="R157" t="n">
+        <v>2.240559345945638</v>
+      </c>
+      <c r="S157" t="n">
+        <v>0.05191929801433606</v>
+      </c>
+      <c r="T157" t="n">
+        <v>0.02700349151234568</v>
+      </c>
+      <c r="U157" t="n">
+        <v>-3.4332275390625e-05</v>
+      </c>
+      <c r="V157" t="n">
+        <v>-0.0002698898315429688</v>
+      </c>
+      <c r="W157" t="n">
+        <v>-2.348423004150391e-05</v>
+      </c>
+      <c r="X157" t="n">
+        <v>-0.06322883513760225</v>
+      </c>
+      <c r="Y157" t="n">
+        <v>0.9483717083930969</v>
+      </c>
+      <c r="Z157" t="n">
+        <v>0.4269917607307434</v>
+      </c>
+      <c r="AA157" t="n">
+        <v>0.6911284603889489</v>
+      </c>
+      <c r="AB157" t="n">
+        <v>-0.04041647911071777</v>
+      </c>
+      <c r="AC157" t="n">
+        <v>-0.0175553560256958</v>
+      </c>
+      <c r="AD157" t="n">
+        <v>0.03275209665298462</v>
+      </c>
+      <c r="AG157" t="n">
+        <v>61</v>
+      </c>
+      <c r="AH157" t="n">
+        <v>0.4809234142303467</v>
+      </c>
+      <c r="BE157" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_g1a_vnhead_plain_wall13000_near2000_split_AG_v1_seed1_20260607_123105</t>
+        </is>
+      </c>
+      <c r="BF157" t="inlineStr">
+        <is>
+          <t>No-Go job 5425；best_wss wss=0.427≈基线 band</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>V3P-G-Baseline-AsymW-a-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>V3P-G-Baseline-AsymW-a-post5463</t>
+        </is>
+      </c>
+      <c r="C158" t="n">
+        <v>1</v>
+      </c>
+      <c r="D158" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K158" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="N158" t="n">
+        <v>185</v>
+      </c>
+      <c r="O158" t="n">
+        <v>0.9032924458880157</v>
+      </c>
+      <c r="P158" t="n">
+        <v>1.078667397258981</v>
+      </c>
+      <c r="Q158" t="n">
+        <v>1.024917140081539</v>
+      </c>
+      <c r="R158" t="n">
+        <v>1.740665317755274</v>
+      </c>
+      <c r="S158" t="n">
+        <v>0.0722431359943799</v>
+      </c>
+      <c r="T158" t="n">
+        <v>0.03542139596193416</v>
+      </c>
+      <c r="U158" t="n">
+        <v>-0.0004887580871582031</v>
+      </c>
+      <c r="V158" t="n">
+        <v>5.960464477539062e-08</v>
+      </c>
+      <c r="W158" t="n">
+        <v>-2.741813659667969e-06</v>
+      </c>
+      <c r="X158" t="n">
+        <v>-0.06888158154521085</v>
+      </c>
+      <c r="Y158" t="n">
+        <v>0.9460028409957886</v>
+      </c>
+      <c r="Z158" t="n">
+        <v>0.4278444051742554</v>
+      </c>
+      <c r="AA158" t="n">
+        <v>0.6998916883310962</v>
+      </c>
+      <c r="AB158" t="n">
+        <v>0.001623153686523438</v>
+      </c>
+      <c r="AC158" t="n">
+        <v>0.003317177295684814</v>
+      </c>
+      <c r="AD158" t="n">
+        <v>0.4079930186271667</v>
+      </c>
+      <c r="AG158" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH158" t="n">
+        <v>0.4980224967002869</v>
+      </c>
+      <c r="BE158" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260608_154606</t>
+        </is>
+      </c>
+      <c r="BF158" t="inlineStr">
+        <is>
+          <t>三 seed 5466/5468/5478；band 0.409–0.437（均值 ~0.425）</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>V3P-G-Baseline-AsymW-a-post5463_seed2</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>V3P-G-Baseline-AsymW-a-post5463</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>2</v>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K159" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="N159" t="n">
+        <v>86</v>
+      </c>
+      <c r="O159" t="n">
+        <v>0.9032924458880157</v>
+      </c>
+      <c r="P159" t="n">
+        <v>1.078667397258981</v>
+      </c>
+      <c r="Q159" t="n">
+        <v>1.024917140081539</v>
+      </c>
+      <c r="R159" t="n">
+        <v>1.740665317755274</v>
+      </c>
+      <c r="S159" t="n">
+        <v>0.08183348625947467</v>
+      </c>
+      <c r="T159" t="n">
+        <v>0.04004677211934157</v>
+      </c>
+      <c r="U159" t="n">
+        <v>-0.0004887580871582031</v>
+      </c>
+      <c r="V159" t="n">
+        <v>5.960464477539062e-08</v>
+      </c>
+      <c r="W159" t="n">
+        <v>-2.741813659667969e-06</v>
+      </c>
+      <c r="X159" t="n">
+        <v>-0.06888158154521085</v>
+      </c>
+      <c r="Y159" t="n">
+        <v>0.9307149052619934</v>
+      </c>
+      <c r="Z159" t="n">
+        <v>0.4373782277107239</v>
+      </c>
+      <c r="AA159" t="n">
+        <v>0.6940360551515788</v>
+      </c>
+      <c r="AB159" t="n">
+        <v>-0.001331567764282227</v>
+      </c>
+      <c r="AC159" t="n">
+        <v>0.006514072418212891</v>
+      </c>
+      <c r="AD159" t="n">
+        <v>0.4078913331031799</v>
+      </c>
+      <c r="AG159" t="n">
+        <v>10</v>
+      </c>
+      <c r="AH159" t="n">
+        <v>0.4947876334190369</v>
+      </c>
+      <c r="BE159" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed2_20260608_154606</t>
+        </is>
+      </c>
+      <c r="BF159" t="inlineStr">
+        <is>
+          <t>三 seed 5466/5468/5478；band 0.409–0.437（均值 ~0.425）</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>V3P-G-58-SSL-Finetune_seed1</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>V3P-G-58-SSL-Finetune</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>1</v>
+      </c>
+      <c r="D160" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K160" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="N160" t="n">
+        <v>98</v>
+      </c>
+      <c r="O160" t="n">
+        <v>0.9032924458880157</v>
+      </c>
+      <c r="P160" t="n">
+        <v>1.078667397258981</v>
+      </c>
+      <c r="Q160" t="n">
+        <v>1.024917140081539</v>
+      </c>
+      <c r="R160" t="n">
+        <v>1.740665317755274</v>
+      </c>
+      <c r="S160" t="n">
+        <v>0.07726986991334266</v>
+      </c>
+      <c r="T160" t="n">
+        <v>0.04678496656378601</v>
+      </c>
+      <c r="U160" t="n">
+        <v>-0.0004887580871582031</v>
+      </c>
+      <c r="V160" t="n">
+        <v>5.960464477539062e-08</v>
+      </c>
+      <c r="W160" t="n">
+        <v>-2.741813659667969e-06</v>
+      </c>
+      <c r="X160" t="n">
+        <v>-0.06888158154521085</v>
+      </c>
+      <c r="Y160" t="n">
+        <v>0.938227117061615</v>
+      </c>
+      <c r="Z160" t="n">
+        <v>0.4400887489318848</v>
+      </c>
+      <c r="AA160" t="n">
+        <v>0.6923622251045014</v>
+      </c>
+      <c r="AB160" t="n">
+        <v>0.02351748943328857</v>
+      </c>
+      <c r="AC160" t="n">
+        <v>0.004679262638092041</v>
+      </c>
+      <c r="AD160" t="n">
+        <v>0.4100866317749023</v>
+      </c>
+      <c r="AG160" t="n">
+        <v>36</v>
+      </c>
+      <c r="AH160" t="n">
+        <v>0.4932488203048706</v>
+      </c>
+      <c r="BE160" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260609_124213</t>
+        </is>
+      </c>
+      <c r="BF160" t="inlineStr">
+        <is>
+          <t>No-Go jobs 5474/5475；wss 0.435–0.440；未达 Go +0.03 vs post5463 band</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>V3P-G-58-SSL-Finetune_seed2</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>V3P-G-58-SSL-Finetune</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>2</v>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K161" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="N161" t="n">
+        <v>164</v>
+      </c>
+      <c r="O161" t="n">
+        <v>0.9032924458880157</v>
+      </c>
+      <c r="P161" t="n">
+        <v>1.078667397258981</v>
+      </c>
+      <c r="Q161" t="n">
+        <v>1.024917140081539</v>
+      </c>
+      <c r="R161" t="n">
+        <v>1.740665317755274</v>
+      </c>
+      <c r="S161" t="n">
+        <v>0.07453990983220472</v>
+      </c>
+      <c r="T161" t="n">
+        <v>0.04368624614197531</v>
+      </c>
+      <c r="U161" t="n">
+        <v>-0.0004887580871582031</v>
+      </c>
+      <c r="V161" t="n">
+        <v>5.960464477539062e-08</v>
+      </c>
+      <c r="W161" t="n">
+        <v>-2.741813659667969e-06</v>
+      </c>
+      <c r="X161" t="n">
+        <v>-0.06888158154521085</v>
+      </c>
+      <c r="Y161" t="n">
+        <v>0.9425148963928223</v>
+      </c>
+      <c r="Z161" t="n">
+        <v>0.4354023337364197</v>
+      </c>
+      <c r="AA161" t="n">
+        <v>0.6952536997857498</v>
+      </c>
+      <c r="AB161" t="n">
+        <v>0.03326809406280518</v>
+      </c>
+      <c r="AC161" t="n">
+        <v>0.006444096565246582</v>
+      </c>
+      <c r="AD161" t="n">
+        <v>0.410913348197937</v>
+      </c>
+      <c r="AG161" t="n">
+        <v>41</v>
+      </c>
+      <c r="AH161" t="n">
+        <v>0.5003484487533569</v>
+      </c>
+      <c r="BE161" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed2_20260609_124213</t>
+        </is>
+      </c>
+      <c r="BF161" t="inlineStr">
+        <is>
+          <t>No-Go jobs 5474/5475；wss 0.435–0.440；未达 Go +0.03 vs post5463 band</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>V3P-G-Baseline-AsymW-a-post5463_seed3</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>V3P-G-Baseline-AsymW-a-post5463</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>3</v>
+      </c>
+      <c r="D162" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K162" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="N162" t="n">
+        <v>131</v>
+      </c>
+      <c r="O162" t="n">
+        <v>0.9032924458880157</v>
+      </c>
+      <c r="P162" t="n">
+        <v>1.078667397258981</v>
+      </c>
+      <c r="Q162" t="n">
+        <v>1.024917140081539</v>
+      </c>
+      <c r="R162" t="n">
+        <v>1.740665317755274</v>
+      </c>
+      <c r="S162" t="n">
+        <v>0.07251228532653449</v>
+      </c>
+      <c r="T162" t="n">
+        <v>0.03659742155349794</v>
+      </c>
+      <c r="U162" t="n">
+        <v>-0.0004887580871582031</v>
+      </c>
+      <c r="V162" t="n">
+        <v>5.960464477539062e-08</v>
+      </c>
+      <c r="W162" t="n">
+        <v>-2.741813659667969e-06</v>
+      </c>
+      <c r="X162" t="n">
+        <v>-0.06888158154521085</v>
+      </c>
+      <c r="Y162" t="n">
+        <v>0.9455997943878174</v>
+      </c>
+      <c r="Z162" t="n">
+        <v>0.4087181687355042</v>
+      </c>
+      <c r="AA162" t="n">
+        <v>0.7114936463600106</v>
+      </c>
+      <c r="AB162" t="n">
+        <v>-0.0004200935363769531</v>
+      </c>
+      <c r="AC162" t="n">
+        <v>0.01253718137741089</v>
+      </c>
+      <c r="AD162" t="n">
+        <v>0.3746001720428467</v>
+      </c>
+      <c r="AG162" t="n">
+        <v>52</v>
+      </c>
+      <c r="AH162" t="n">
+        <v>0.4958834648132324</v>
+      </c>
+      <c r="BE162" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed3_20260610_003850</t>
+        </is>
+      </c>
+      <c r="BF162" t="inlineStr">
+        <is>
+          <t>三 seed 5466/5468/5478；band 0.409–0.437（均值 ~0.425）</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>V3P-I2-PC-Intrinsic_seed1</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>V3P-I2-PC-Intrinsic</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>1</v>
+      </c>
+      <c r="D163" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K163" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="N163" t="n">
+        <v>109</v>
+      </c>
+      <c r="O163" t="n">
+        <v>0.9032924458880157</v>
+      </c>
+      <c r="P163" t="n">
+        <v>1.078667397258981</v>
+      </c>
+      <c r="Q163" t="n">
+        <v>1.024917140081539</v>
+      </c>
+      <c r="R163" t="n">
+        <v>1.740665317755274</v>
+      </c>
+      <c r="S163" t="n">
+        <v>0.07905139786882602</v>
+      </c>
+      <c r="T163" t="n">
+        <v>0.03840403485082305</v>
+      </c>
+      <c r="U163" t="n">
+        <v>-0.0004887580871582031</v>
+      </c>
+      <c r="V163" t="n">
+        <v>5.960464477539062e-08</v>
+      </c>
+      <c r="W163" t="n">
+        <v>-2.741813659667969e-06</v>
+      </c>
+      <c r="X163" t="n">
+        <v>-0.06888158154521085</v>
+      </c>
+      <c r="Y163" t="n">
+        <v>0.9353458285331726</v>
+      </c>
+      <c r="Z163" t="n">
+        <v>0.4174727201461792</v>
+      </c>
+      <c r="AA163" t="n">
+        <v>0.7062068120065579</v>
+      </c>
+      <c r="AG163" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH163" t="n">
+        <v>0.2526676942949185</v>
+      </c>
+      <c r="BE163" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_i2pc_intrinsic_geom_pw_asymw_wall13000_near2000_split_AG_v1_seed1_20260618_143615</t>
+        </is>
+      </c>
+      <c r="BF163" t="inlineStr">
+        <is>
+          <t>No-Go job 5741；best_wss wss=0.417；local frame 4D 未破 band</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>V3P-I6-diag-AsymW-a-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>V3P-I6-diag-AsymW-a-post5463</t>
+        </is>
+      </c>
+      <c r="C164" t="n">
+        <v>1</v>
+      </c>
+      <c r="D164" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K164" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="N164" t="n">
+        <v>163</v>
+      </c>
+      <c r="O164" t="n">
+        <v>0.9032924458880157</v>
+      </c>
+      <c r="P164" t="n">
+        <v>1.078667397258981</v>
+      </c>
+      <c r="Q164" t="n">
+        <v>1.024917140081539</v>
+      </c>
+      <c r="R164" t="n">
+        <v>1.740665317755274</v>
+      </c>
+      <c r="S164" t="n">
+        <v>0.07658495723385446</v>
+      </c>
+      <c r="T164" t="n">
+        <v>0.03733061985596708</v>
+      </c>
+      <c r="U164" t="n">
+        <v>-0.0004887580871582031</v>
+      </c>
+      <c r="V164" t="n">
+        <v>5.960464477539062e-08</v>
+      </c>
+      <c r="W164" t="n">
+        <v>-2.741813659667969e-06</v>
+      </c>
+      <c r="X164" t="n">
+        <v>-0.06888158154521085</v>
+      </c>
+      <c r="Y164" t="n">
+        <v>0.9393173456192017</v>
+      </c>
+      <c r="Z164" t="n">
+        <v>0.4286386370658875</v>
+      </c>
+      <c r="AA164" t="n">
+        <v>0.6994057636884691</v>
+      </c>
+      <c r="AB164" t="n">
+        <v>0.001799464225769043</v>
+      </c>
+      <c r="AC164" t="n">
+        <v>0.003979504108428955</v>
+      </c>
+      <c r="AD164" t="n">
+        <v>0.4081660509109497</v>
+      </c>
+      <c r="AG164" t="n">
+        <v>6</v>
+      </c>
+      <c r="AH164" t="n">
+        <v>0.4907243847846985</v>
+      </c>
+      <c r="BE164" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_i6diag_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260619_174001</t>
+        </is>
+      </c>
+      <c r="BF164" t="inlineStr">
+        <is>
+          <t>平台期带宽参考 job 5463/I6-diag；best_wss wss=0.429 · r2_p=0.930</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>V3P-I6-a-AsymW-a-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>V3P-I6-a-AsymW-a-post5463</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>1</v>
+      </c>
+      <c r="D165" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K165" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="N165" t="n">
+        <v>33</v>
+      </c>
+      <c r="O165" t="n">
+        <v>0.9032924458880157</v>
+      </c>
+      <c r="P165" t="n">
+        <v>1.078667397258981</v>
+      </c>
+      <c r="Q165" t="n">
+        <v>1.024917140081539</v>
+      </c>
+      <c r="R165" t="n">
+        <v>1.740665317755274</v>
+      </c>
+      <c r="S165" t="n">
+        <v>0.07567738934602893</v>
+      </c>
+      <c r="T165" t="n">
+        <v>0.04453175154320987</v>
+      </c>
+      <c r="U165" t="n">
+        <v>-0.0004887580871582031</v>
+      </c>
+      <c r="V165" t="n">
+        <v>5.960464477539062e-08</v>
+      </c>
+      <c r="W165" t="n">
+        <v>-2.741813659667969e-06</v>
+      </c>
+      <c r="X165" t="n">
+        <v>-0.06888158154521085</v>
+      </c>
+      <c r="Y165" t="n">
+        <v>0.940747082233429</v>
+      </c>
+      <c r="Z165" t="n">
+        <v>0.4457049965858459</v>
+      </c>
+      <c r="AA165" t="n">
+        <v>0.6888810724299982</v>
+      </c>
+      <c r="AB165" t="n">
+        <v>-0.0001618862152099609</v>
+      </c>
+      <c r="AC165" t="n">
+        <v>-0.000516057014465332</v>
+      </c>
+      <c r="AD165" t="n">
+        <v>0.4160026907920837</v>
+      </c>
+      <c r="AG165" t="n">
+        <v>12</v>
+      </c>
+      <c r="AH165" t="n">
+        <v>0.4635753035545349</v>
+      </c>
+      <c r="BE165" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_i6a_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260625_154438</t>
+        </is>
+      </c>
+      <c r="BF165" t="inlineStr">
+        <is>
+          <t>Go job 5810；best_wss wss=0.446（+0.017 vs I6-diag）；未扩 seed</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>V3P-M-E-WSSOnly-AsymW-a-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>V3P-M-E-WSSOnly-AsymW-a-post5463</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>1</v>
+      </c>
+      <c r="D166" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K166" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M166" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="N166" t="n">
+        <v>13</v>
+      </c>
+      <c r="O166" t="n">
+        <v>1.020887514309205</v>
+      </c>
+      <c r="P166" t="n">
+        <v>1.147455630457367</v>
+      </c>
+      <c r="Q166" t="n">
+        <v>1.063679894373995</v>
+      </c>
+      <c r="R166" t="n">
+        <v>1.704777096253831</v>
+      </c>
+      <c r="S166" t="n">
+        <v>0.3554859596238816</v>
+      </c>
+      <c r="T166" t="n">
+        <v>0.2977987911522634</v>
+      </c>
+      <c r="U166" t="n">
+        <v>-0.2779422998428345</v>
+      </c>
+      <c r="V166" t="n">
+        <v>-0.1316096782684326</v>
+      </c>
+      <c r="W166" t="n">
+        <v>-0.07707405090332031</v>
+      </c>
+      <c r="X166" t="n">
+        <v>-0.02526054578139481</v>
+      </c>
+      <c r="Y166" t="n">
+        <v>-0.3074421882629395</v>
+      </c>
+      <c r="Z166" t="n">
+        <v>0.4105274081230164</v>
+      </c>
+      <c r="AA166" t="n">
+        <v>0.7104042785347154</v>
+      </c>
+      <c r="AB166" t="n">
+        <v>0.03176093101501465</v>
+      </c>
+      <c r="AC166" t="n">
+        <v>0.02013051509857178</v>
+      </c>
+      <c r="AD166" t="n">
+        <v>0.3896239995956421</v>
+      </c>
+      <c r="AG166" t="n">
+        <v>25</v>
+      </c>
+      <c r="AH166" t="n">
+        <v>0.4636592864990234</v>
+      </c>
+      <c r="BE166" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_mewssonly_localpool_main01_geom_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260625_155102</t>
+        </is>
+      </c>
+      <c r="BF166" t="inlineStr">
+        <is>
+          <t>No-Go job 5811；WSS-only；wss=0.411 但 r2_p≈−0.41</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>V3P-M-E-PWeak-AsymW-a-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>V3P-M-E-PWeak-AsymW-a-post5463</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>1</v>
+      </c>
+      <c r="D167" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K167" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="N167" t="n">
+        <v>151</v>
+      </c>
+      <c r="O167" t="n">
+        <v>0.9032924458880157</v>
+      </c>
+      <c r="P167" t="n">
+        <v>1.078667397258981</v>
+      </c>
+      <c r="Q167" t="n">
+        <v>1.024917140081539</v>
+      </c>
+      <c r="R167" t="n">
+        <v>1.740665317755274</v>
+      </c>
+      <c r="S167" t="n">
+        <v>0.07112423528431647</v>
+      </c>
+      <c r="T167" t="n">
+        <v>0.03949427404835391</v>
+      </c>
+      <c r="U167" t="n">
+        <v>-0.0004887580871582031</v>
+      </c>
+      <c r="V167" t="n">
+        <v>5.960464477539062e-08</v>
+      </c>
+      <c r="W167" t="n">
+        <v>-2.741813659667969e-06</v>
+      </c>
+      <c r="X167" t="n">
+        <v>-0.06888158154521085</v>
+      </c>
+      <c r="Y167" t="n">
+        <v>0.9476625323295593</v>
+      </c>
+      <c r="Z167" t="n">
+        <v>0.4112195372581482</v>
+      </c>
+      <c r="AA167" t="n">
+        <v>0.7099871132363346</v>
+      </c>
+      <c r="AB167" t="n">
+        <v>0.03429305553436279</v>
+      </c>
+      <c r="AC167" t="n">
+        <v>0.03664183616638184</v>
+      </c>
+      <c r="AD167" t="n">
+        <v>0.39704829454422</v>
+      </c>
+      <c r="AG167" t="n">
+        <v>70</v>
+      </c>
+      <c r="AH167" t="n">
+        <v>0.4922247529029846</v>
+      </c>
+      <c r="BE167" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_mepweak_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260625_155102</t>
+        </is>
+      </c>
+      <c r="BF167" t="inlineStr">
+        <is>
+          <t>No-Go job 5812；弱压力 λ；best_wss wss=0.411</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>V3P-M-E-EJ-PGradBridge-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>V3P-M-E-EJ-PGradBridge-post5463</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>1</v>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K168" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M168" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="N168" t="n">
+        <v>77</v>
+      </c>
+      <c r="O168" t="n">
+        <v>0.9032924458880157</v>
+      </c>
+      <c r="P168" t="n">
+        <v>1.078667397258981</v>
+      </c>
+      <c r="Q168" t="n">
+        <v>1.024917140081539</v>
+      </c>
+      <c r="R168" t="n">
+        <v>1.740665317755274</v>
+      </c>
+      <c r="S168" t="n">
+        <v>0.07770820921447738</v>
+      </c>
+      <c r="T168" t="n">
+        <v>0.03820983153292181</v>
+      </c>
+      <c r="U168" t="n">
+        <v>-0.0004887580871582031</v>
+      </c>
+      <c r="V168" t="n">
+        <v>5.960464477539062e-08</v>
+      </c>
+      <c r="W168" t="n">
+        <v>-2.741813659667969e-06</v>
+      </c>
+      <c r="X168" t="n">
+        <v>-0.06888158154521085</v>
+      </c>
+      <c r="Y168" t="n">
+        <v>0.9375242590904236</v>
+      </c>
+      <c r="Z168" t="n">
+        <v>0.4008861184120178</v>
+      </c>
+      <c r="AA168" t="n">
+        <v>0.7161903365019455</v>
+      </c>
+      <c r="AB168" t="n">
+        <v>0.003787219524383545</v>
+      </c>
+      <c r="AC168" t="n">
+        <v>0.01260608434677124</v>
+      </c>
+      <c r="AD168" t="n">
+        <v>0.3835007548332214</v>
+      </c>
+      <c r="AG168" t="n">
+        <v>56</v>
+      </c>
+      <c r="AH168" t="n">
+        <v>0.4879887104034424</v>
+      </c>
+      <c r="BE168" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_me_ej_pgradbridge_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260629_154517</t>
+        </is>
+      </c>
+      <c r="BF168" t="inlineStr">
+        <is>
+          <t>No-Go job 5854；rich pgrad context；best_wss wss=0.401</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>V3P-J4-V3Dlite-MixedProbe-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>V3P-J4-V3Dlite-MixedProbe-post5463</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>1</v>
+      </c>
+      <c r="D169" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K169" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr">
+        <is>
+          <t>split_AG_v3lite_v1</t>
+        </is>
+      </c>
+      <c r="N169" t="n">
+        <v>39</v>
+      </c>
+      <c r="O169" t="n">
+        <v>0.9032924458880157</v>
+      </c>
+      <c r="P169" t="n">
+        <v>1.078667397258981</v>
+      </c>
+      <c r="Q169" t="n">
+        <v>1.024917140081539</v>
+      </c>
+      <c r="R169" t="n">
+        <v>1.740665317755274</v>
+      </c>
+      <c r="S169" t="n">
+        <v>0.07581888026188903</v>
+      </c>
+      <c r="T169" t="n">
+        <v>0.04064371784979424</v>
+      </c>
+      <c r="U169" t="n">
+        <v>-0.0004887580871582031</v>
+      </c>
+      <c r="V169" t="n">
+        <v>5.960464477539062e-08</v>
+      </c>
+      <c r="W169" t="n">
+        <v>-2.741813659667969e-06</v>
+      </c>
+      <c r="X169" t="n">
+        <v>-0.06888158154521085</v>
+      </c>
+      <c r="Y169" t="n">
+        <v>0.9405252933502197</v>
+      </c>
+      <c r="Z169" t="n">
+        <v>0.4231371879577637</v>
+      </c>
+      <c r="AA169" t="n">
+        <v>0.7027648537707556</v>
+      </c>
+      <c r="AB169" t="n">
+        <v>0.0004634857177734375</v>
+      </c>
+      <c r="AC169" t="n">
+        <v>0.006696105003356934</v>
+      </c>
+      <c r="AD169" t="n">
+        <v>0.3975040912628174</v>
+      </c>
+      <c r="AG169" t="n">
+        <v>29</v>
+      </c>
+      <c r="AH169" t="n">
+        <v>0.4843106865882874</v>
+      </c>
+      <c r="BE169" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_j4v3dlite_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v3lite_v1_seed1_20260630_131820</t>
+        </is>
+      </c>
+      <c r="BF169" t="inlineStr">
+        <is>
+          <t>No-Go job 5872；+1 ZHAO；best_wss wss=0.423（Δi6 −0.006）</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>V3P-J5-ActiveData-MixedProbe-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>V3P-J5-ActiveData-MixedProbe-post5463</t>
+        </is>
+      </c>
+      <c r="C170" t="n">
+        <v>1</v>
+      </c>
+      <c r="D170" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_wall</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K170" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr">
+        <is>
+          <t>split_AG_active_v2_j5</t>
+        </is>
+      </c>
+      <c r="N170" t="n">
+        <v>37</v>
+      </c>
+      <c r="O170" t="n">
+        <v>0.9032923604666244</v>
+      </c>
+      <c r="P170" t="n">
+        <v>1.078667158815069</v>
+      </c>
+      <c r="Q170" t="n">
+        <v>1.024916989512295</v>
+      </c>
+      <c r="R170" t="n">
+        <v>1.740665317755274</v>
+      </c>
+      <c r="S170" t="n">
+        <v>0.06819546983840995</v>
+      </c>
+      <c r="T170" t="n">
+        <v>0.03806694958847737</v>
+      </c>
+      <c r="U170" t="n">
+        <v>-0.0004903078079223633</v>
+      </c>
+      <c r="V170" t="n">
+        <v>1.788139343261719e-07</v>
+      </c>
+      <c r="W170" t="n">
+        <v>-2.86102294921875e-06</v>
+      </c>
+      <c r="X170" t="n">
+        <v>-0.06888158154521129</v>
+      </c>
+      <c r="Y170" t="n">
+        <v>0.9518840312957764</v>
+      </c>
+      <c r="Z170" t="n">
+        <v>0.4329603314399719</v>
+      </c>
+      <c r="AA170" t="n">
+        <v>0.6967558508006809</v>
+      </c>
+      <c r="AB170" t="n">
+        <v>0.004196524620056152</v>
+      </c>
+      <c r="AC170" t="n">
+        <v>0.005350887775421143</v>
+      </c>
+      <c r="AD170" t="n">
+        <v>0.408894419670105</v>
+      </c>
+      <c r="AG170" t="n">
+        <v>39</v>
+      </c>
+      <c r="AH170" t="n">
+        <v>0.4844380617141724</v>
+      </c>
+      <c r="BE170" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_j5activedata_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_active_v2_j5_seed1_20260701_002549</t>
+        </is>
+      </c>
+      <c r="BF170" t="inlineStr">
+        <is>
+          <t>弱 No-Go jobs 5881–5883；+6 AAA；wss=0.433（Δi6 +0.004）；Go 0.459 未过</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>V3P-K1-BranchFeat-MixedProbe-post5463_seed1</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>V3P-K1-BranchFeat-MixedProbe-post5463</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>1</v>
+      </c>
+      <c r="D171" t="inlineStr">
+        <is>
+          <t>pointnext</t>
+        </is>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>coord_t_bc_geom_g01_wall</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K171" t="inlineStr">
+        <is>
+          <t>mlp2</t>
+        </is>
+      </c>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>wall13000_near2000</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr">
+        <is>
+          <t>split_AG_v1</t>
+        </is>
+      </c>
+      <c r="N171" t="n">
+        <v>29</v>
+      </c>
+      <c r="O171" t="n">
+        <v>0.9032924458880157</v>
+      </c>
+      <c r="P171" t="n">
+        <v>1.078667397258981</v>
+      </c>
+      <c r="Q171" t="n">
+        <v>1.024917140081539</v>
+      </c>
+      <c r="R171" t="n">
+        <v>1.740665317755274</v>
+      </c>
+      <c r="S171" t="n">
+        <v>0.07864104003870588</v>
+      </c>
+      <c r="T171" t="n">
+        <v>0.0423220100308642</v>
+      </c>
+      <c r="U171" t="n">
+        <v>-0.0004887580871582031</v>
+      </c>
+      <c r="V171" t="n">
+        <v>5.960464477539062e-08</v>
+      </c>
+      <c r="W171" t="n">
+        <v>-2.741813659667969e-06</v>
+      </c>
+      <c r="X171" t="n">
+        <v>-0.06888158154521085</v>
+      </c>
+      <c r="Y171" t="n">
+        <v>0.9360153079032898</v>
+      </c>
+      <c r="Z171" t="n">
+        <v>0.3998472094535828</v>
+      </c>
+      <c r="AA171" t="n">
+        <v>0.7168110315999805</v>
+      </c>
+      <c r="AB171" t="n">
+        <v>0.003674745559692383</v>
+      </c>
+      <c r="AC171" t="n">
+        <v>0.006487429141998291</v>
+      </c>
+      <c r="AD171" t="n">
+        <v>0.3778122067451477</v>
+      </c>
+      <c r="AG171" t="n">
+        <v>38</v>
+      </c>
+      <c r="AH171" t="n">
+        <v>0.4774236679077148</v>
+      </c>
+      <c r="BE171" t="inlineStr">
+        <is>
+          <t>outputs/field/field_v3_pointnext_k1branchfeat_localpool_main01_geom_pw_asymw_a_wall13000_near2000_split_AG_v1_seed1_20260701_150937</t>
+        </is>
+      </c>
+      <c r="BF171" t="inlineStr">
+        <is>
+          <t>No-Go job 5886；branch 特征短训；best_wss wss=0.400（低于 I6-diag）</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>